<commit_message>
update: update to the latest version
</commit_message>
<xml_diff>
--- a/Modif_fichier_preset/test5_change.xlsx
+++ b/Modif_fichier_preset/test5_change.xlsx
@@ -1059,10 +1059,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>149.29</v>
+        <v>80.7</v>
       </c>
       <c r="C2" t="n">
-        <v>58.48</v>
+        <v>77.13</v>
       </c>
     </row>
     <row r="3">
@@ -1154,10 +1154,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-69.44</v>
+        <v>-85.34</v>
       </c>
       <c r="C2" t="n">
-        <v>-17.45</v>
+        <v>-25.71</v>
       </c>
     </row>
     <row r="3">

</xml_diff>